<commit_message>
Update research staff and Valerie publications
</commit_message>
<xml_diff>
--- a/research_staff/working_papers.xlsx
+++ b/research_staff/working_papers.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Working papers" sheetId="1" r:id="Re27f88cb6dfd4713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Working papers" sheetId="1" r:id="Re1ddcb289f7e4766"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="12">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -96,6 +96,9 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -107,7 +110,7 @@
         <x:color rgb="FF7A4F00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -117,7 +120,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Personal_Website_Working_Papers" displayName="Personal_Website_Working_Papers" ref="A1:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Personal_Website_Working_Papers" displayName="Personal_Website_Working_Papers" ref="A1:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Staff member"/>
     <x:tableColumn id="2" name="Title"/>
@@ -749,13 +752,57 @@
         <x:v>Review</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A19" s="12" t="str">
+        <x:v>Valerie Lechene</x:v>
+      </x:c>
+      <x:c r="B19" s="12" t="str">
+        <x:v>Gender inequality in expenditure: Great Britain 1978 to 2019</x:v>
+      </x:c>
+      <x:c r="C19" s="12" t="str">
+        <x:v>https://ifs.org.uk/publications/gender-inequality-expenditure-great-britain-1978-2019</x:v>
+      </x:c>
+      <x:c r="D19" s="12" t="str">
+        <x:v>Working papers and current research</x:v>
+      </x:c>
+      <x:c r="E19" s="12" t="str">
+        <x:v>https://www.valerielechene.com/home/research</x:v>
+      </x:c>
+      <x:c r="F19" s="12" t="str">
+        <x:v>Personal webpage</x:v>
+      </x:c>
+      <x:c r="G19" s="12" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A20" s="12" t="str">
+        <x:v>Valerie Lechene</x:v>
+      </x:c>
+      <x:c r="B20" s="12" t="str">
+        <x:v>Documenting individual poverty in South Africa and Ethiopia</x:v>
+      </x:c>
+      <x:c r="C20" s="12" t="str"/>
+      <x:c r="D20" s="12" t="str">
+        <x:v>Working papers and current research</x:v>
+      </x:c>
+      <x:c r="E20" s="12" t="str">
+        <x:v>https://www.valerielechene.com/home/research</x:v>
+      </x:c>
+      <x:c r="F20" s="12" t="str">
+        <x:v>Personal webpage</x:v>
+      </x:c>
+      <x:c r="G20" s="12" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="G2:G18">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Review"/>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47ee021dae994e53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd577fafe8fd342f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>